<commit_message>
Updated the code for APA diagram
</commit_message>
<xml_diff>
--- a/output/raster/day/deltaT/deltaT_20210108_accuracy.xlsx
+++ b/output/raster/day/deltaT/deltaT_20210108_accuracy.xlsx
@@ -411,16 +411,16 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>-0.01978645575462738</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>0.02741102798075643</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>0.07374938884315838</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>0.1737361454672</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -428,16 +428,16 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>-0.01978645575462738</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>0.02741102798075643</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>0.07374938884315838</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>0.1737361454672</v>
       </c>
     </row>
   </sheetData>

</xml_diff>